<commit_message>
✨ feat(playwright): IOL formula calculation script
</commit_message>
<xml_diff>
--- a/Kanedata.xlsx
+++ b/Kanedata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\yokam\PycharmProjects\BarrettAutomate\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4582BDF1-9A77-45D1-BC27-98FD737DE3A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0746B23F-F006-47BB-9694-28C3D194E3A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6780" yWindow="336" windowWidth="17196" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5100" yWindow="384" windowWidth="17196" windowHeight="12240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="36" r:id="rId1"/>

</xml_diff>